<commit_message>
Set up starter code
Remove uunnecessarycode down to sskeletoncode.
</commit_message>
<xml_diff>
--- a/Misc files/Capstone Schedule.xlsx
+++ b/Misc files/Capstone Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/bryce_e_rooney_civ_us_navy_mil/Documents/Documents/School stuff/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yayal\Documents\Bryce\WES-CAPSTONE\Misc files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{72A988FC-158D-4AB4-AB94-8415EF19A469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1FFE42D-72E5-4E3D-96EF-63AC4CCAAADB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01868711-D0CC-4E23-9B76-E4955F5DA0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7410" yWindow="1680" windowWidth="32790" windowHeight="18825" xr2:uid="{9E7B8A6A-42F7-4783-B41C-E02948B47874}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="10020" xr2:uid="{9E7B8A6A-42F7-4783-B41C-E02948B47874}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Week 2</t>
   </si>
@@ -126,13 +126,16 @@
   </si>
   <si>
     <t>Complete</t>
+  </si>
+  <si>
+    <t>Milestone Updates</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,7 +319,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
@@ -326,7 +329,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3" applyBorder="1"/>
@@ -362,10 +364,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -685,16 +683,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FA40F8A-DE14-4A53-9DE9-CC33AFA0ED4A}">
-  <dimension ref="B2:M27"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="B2:M32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="36.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="10.125" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="15" thickBot="1"/>
-    <row r="3" spans="2:13">
+    <row r="2" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
@@ -729,43 +727,43 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="15" thickBot="1">
-      <c r="C4" s="20">
+    <row r="4" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="19">
         <v>46115</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="20">
         <v>46122</v>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="20">
         <v>46129</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="20">
         <v>46136</v>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="20">
         <v>46143</v>
       </c>
-      <c r="H4" s="21">
+      <c r="H4" s="20">
         <v>46150</v>
       </c>
-      <c r="I4" s="21">
+      <c r="I4" s="20">
         <v>46157</v>
       </c>
-      <c r="J4" s="21">
+      <c r="J4" s="20">
         <v>46164</v>
       </c>
-      <c r="K4" s="21">
+      <c r="K4" s="20">
         <v>46171</v>
       </c>
-      <c r="L4" s="21">
+      <c r="L4" s="20">
         <v>46178</v>
       </c>
-      <c r="M4" s="22">
+      <c r="M4" s="21">
         <v>46183</v>
       </c>
     </row>
-    <row r="5" spans="2:13">
-      <c r="B5" s="17" t="s">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B5" s="16" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="6"/>
@@ -780,272 +778,130 @@
       <c r="L5" s="7"/>
       <c r="M5" s="8"/>
     </row>
-    <row r="6" spans="2:13">
-      <c r="B6" s="18" t="s">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="11"/>
-    </row>
-    <row r="7" spans="2:13">
-      <c r="B7" s="18"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="11"/>
-    </row>
-    <row r="8" spans="2:13">
-      <c r="B8" s="18" t="s">
+      <c r="D6" s="9"/>
+      <c r="M6" s="10"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="17"/>
+      <c r="M7" s="10"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B8" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="11"/>
-    </row>
-    <row r="9" spans="2:13">
-      <c r="B9" s="18" t="s">
+      <c r="E8" s="11"/>
+      <c r="M8" s="10"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B9" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="11"/>
-    </row>
-    <row r="10" spans="2:13">
-      <c r="B10" s="18" t="s">
+      <c r="E9" s="11"/>
+      <c r="M9" s="10"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B10" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="11"/>
-    </row>
-    <row r="11" spans="2:13">
-      <c r="B11" s="18" t="s">
+      <c r="F10" s="11"/>
+      <c r="M10" s="10"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B11" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="11"/>
-    </row>
-    <row r="12" spans="2:13">
-      <c r="B12" s="18" t="s">
+      <c r="G11" s="11"/>
+      <c r="M11" s="10"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B12" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="11"/>
-    </row>
-    <row r="13" spans="2:13">
-      <c r="B13" s="18" t="s">
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="M12" s="10"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B13" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="11"/>
-    </row>
-    <row r="14" spans="2:13">
-      <c r="B14" s="18"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="11"/>
-    </row>
-    <row r="15" spans="2:13">
-      <c r="B15" s="18" t="s">
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="M13" s="10"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B14" s="17"/>
+      <c r="M14" s="10"/>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B15" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="11"/>
-    </row>
-    <row r="16" spans="2:13">
-      <c r="B16" s="18" t="s">
+      <c r="H15" s="13"/>
+      <c r="M15" s="10"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B16" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="11"/>
-    </row>
-    <row r="17" spans="2:13">
-      <c r="B17" s="18"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="11"/>
-    </row>
-    <row r="18" spans="2:13">
-      <c r="B18" s="18" t="s">
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="M16" s="10"/>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B17" s="17"/>
+      <c r="M17" s="10"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B18" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="11"/>
-    </row>
-    <row r="19" spans="2:13">
-      <c r="B19" s="18" t="s">
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="M18" s="10"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B19" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="11"/>
-    </row>
-    <row r="20" spans="2:13">
-      <c r="B20" s="18"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="11"/>
-    </row>
-    <row r="21" spans="2:13">
-      <c r="B21" s="18" t="s">
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="M19" s="10"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B20" s="17"/>
+      <c r="M20" s="10"/>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B21" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="11"/>
-    </row>
-    <row r="22" spans="2:13" ht="15" thickBot="1">
-      <c r="B22" s="19" t="s">
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="10"/>
+    </row>
+    <row r="22" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="16"/>
-    </row>
-    <row r="24" spans="2:13">
-      <c r="B24" s="23" t="s">
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="15"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B24" s="22" t="s">
         <v>25</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1053,23 +909,28 @@
       </c>
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="2:13">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C25" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="2:13">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C26" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D26" s="4"/>
     </row>
-    <row r="27" spans="2:13">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C27" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D27" s="2"/>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Debug Ready to Test
Made dedicated Transmission and ACK freq channels. TxandListenForAck was receiving own TX when on the 1 freq channel.

Fixed some ACK logic and prints.
</commit_message>
<xml_diff>
--- a/Misc files/Capstone Schedule.xlsx
+++ b/Misc files/Capstone Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yayal\Documents\Bryce\WES-CAPSTONE\Misc files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Bryce\Documents\_Personal\School\WES-CAPSTONE\Misc files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01868711-D0CC-4E23-9B76-E4955F5DA0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C07A78-4525-4CF4-A130-439C1436A7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="10020" xr2:uid="{9E7B8A6A-42F7-4783-B41C-E02948B47874}"/>
+    <workbookView xWindow="15600" yWindow="4215" windowWidth="17130" windowHeight="13485" xr2:uid="{9E7B8A6A-42F7-4783-B41C-E02948B47874}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="34">
   <si>
     <t>Week 2</t>
   </si>
@@ -128,14 +128,23 @@
     <t>Complete</t>
   </si>
   <si>
-    <t>Milestone Updates</t>
+    <t>Update:</t>
+  </si>
+  <si>
+    <t>&lt;---Moved Left</t>
+  </si>
+  <si>
+    <t>Potential Extension</t>
+  </si>
+  <si>
+    <t>Added</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +168,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -319,7 +336,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
@@ -345,6 +362,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="40% - Accent4" xfId="3" builtinId="43"/>
@@ -683,23 +704,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FA40F8A-DE14-4A53-9DE9-CC33AFA0ED4A}">
-  <dimension ref="B2:M32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:M54"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="36.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.85546875" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D2" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="26">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="16" t="s">
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
@@ -727,14 +755,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C4" s="19">
         <v>46115</v>
       </c>
       <c r="D4" s="20">
         <v>46122</v>
       </c>
-      <c r="E4" s="20">
+      <c r="E4" s="23">
         <v>46129</v>
       </c>
       <c r="F4" s="20">
@@ -762,13 +790,13 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="16" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+      <c r="E5" s="16"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -778,119 +806,133 @@
       <c r="L5" s="7"/>
       <c r="M5" s="8"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="17" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="9"/>
+      <c r="E6" s="17"/>
       <c r="M6" s="10"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="17"/>
+      <c r="E7" s="17"/>
       <c r="M7" s="10"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="11"/>
+      <c r="E8" s="24"/>
       <c r="M8" s="10"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="11"/>
+      <c r="E9" s="24"/>
       <c r="M9" s="10"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="17" t="s">
         <v>20</v>
       </c>
+      <c r="E10" s="17"/>
       <c r="F10" s="11"/>
       <c r="M10" s="10"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" s="17" t="s">
         <v>19</v>
       </c>
+      <c r="E11" s="17"/>
       <c r="G11" s="11"/>
       <c r="M11" s="10"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="17" t="s">
         <v>18</v>
       </c>
+      <c r="E12" s="17"/>
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
       <c r="M12" s="10"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="17" t="s">
         <v>22</v>
       </c>
+      <c r="E13" s="17"/>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
       <c r="M13" s="10"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="17"/>
+      <c r="E14" s="17"/>
       <c r="M14" s="10"/>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" s="17" t="s">
         <v>11</v>
       </c>
+      <c r="E15" s="17"/>
       <c r="H15" s="13"/>
       <c r="M15" s="10"/>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="17" t="s">
         <v>21</v>
       </c>
+      <c r="E16" s="17"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="M16" s="10"/>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="17"/>
+      <c r="E17" s="17"/>
       <c r="M17" s="10"/>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" s="17" t="s">
         <v>24</v>
       </c>
+      <c r="E18" s="17"/>
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
       <c r="M18" s="10"/>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" s="17" t="s">
         <v>23</v>
       </c>
+      <c r="E19" s="17"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
       <c r="M19" s="10"/>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20" s="17"/>
+      <c r="E20" s="17"/>
       <c r="M20" s="10"/>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" s="17" t="s">
         <v>12</v>
       </c>
+      <c r="E21" s="17"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
       <c r="M21" s="10"/>
     </row>
-    <row r="22" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
+      <c r="E22" s="18"/>
       <c r="F22" s="14"/>
       <c r="G22" s="14"/>
       <c r="H22" s="14"/>
@@ -900,7 +942,7 @@
       <c r="L22" s="14"/>
       <c r="M22" s="15"/>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B24" s="22" t="s">
         <v>25</v>
       </c>
@@ -909,28 +951,292 @@
       </c>
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C25" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C26" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D26" s="4"/>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C27" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B32" t="s">
+    <row r="29" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F29" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="G29" s="26">
+        <v>46141</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C30" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M30" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C31" s="19">
+        <v>46115</v>
+      </c>
+      <c r="D31" s="20">
+        <v>46122</v>
+      </c>
+      <c r="E31" s="20">
+        <v>46129</v>
+      </c>
+      <c r="F31" s="20">
+        <v>46136</v>
+      </c>
+      <c r="G31" s="23">
+        <v>46143</v>
+      </c>
+      <c r="H31" s="20">
+        <v>46150</v>
+      </c>
+      <c r="I31" s="20">
+        <v>46157</v>
+      </c>
+      <c r="J31" s="20">
+        <v>46164</v>
+      </c>
+      <c r="K31" s="20">
+        <v>46171</v>
+      </c>
+      <c r="L31" s="20">
+        <v>46178</v>
+      </c>
+      <c r="M31" s="21">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B32" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="6"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="7"/>
+      <c r="L32" s="7"/>
+      <c r="M32" s="8"/>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B33" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="G33" s="17"/>
+      <c r="M33" s="10"/>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="M34" s="10"/>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B35" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="E35" s="9"/>
+      <c r="G35" s="17"/>
+      <c r="M35" s="10"/>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B36" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="9"/>
+      <c r="G36" s="17"/>
+      <c r="M36" s="10"/>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B37" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F37" s="9"/>
+      <c r="G37" s="17"/>
+      <c r="M37" s="10"/>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B38" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="9"/>
+      <c r="M38" s="10"/>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B39" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="M39" s="10"/>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B40" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="M40" s="10"/>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B41" s="17"/>
+      <c r="G41" s="17"/>
+      <c r="M41" s="10"/>
+    </row>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B42" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" s="17"/>
+      <c r="H42" s="13"/>
+      <c r="M42" s="10"/>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B43" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G43" s="13"/>
+      <c r="I43" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="M43" s="10"/>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="M44" s="10"/>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B45" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="G45" s="17"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
+      <c r="M45" s="10"/>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B46" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="G46" s="17"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12"/>
+      <c r="J46" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="M46" s="10"/>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B47" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G47" s="17"/>
+      <c r="K47" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L47" s="3"/>
+      <c r="M47" s="10"/>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B48" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="17"/>
+      <c r="K48" s="13"/>
+      <c r="L48" s="13"/>
+      <c r="M48" s="10"/>
+    </row>
+    <row r="49" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
+      <c r="J49" s="14"/>
+      <c r="K49" s="14"/>
+      <c r="L49" s="14"/>
+      <c r="M49" s="15"/>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B51" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D51" s="1"/>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C52" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="3"/>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C53" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D53" s="4"/>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C54" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
mid quarter update work
</commit_message>
<xml_diff>
--- a/Misc files/Capstone Schedule.xlsx
+++ b/Misc files/Capstone Schedule.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Bryce\Documents\_Personal\School\WES-CAPSTONE\Misc files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yayal\Documents\Bryce\WES-CAPSTONE\Misc files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06FD082A-AACD-4EC2-8CFA-599A34146AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E1CE527-802E-4F8E-8063-97744D82551E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12510" yWindow="7515" windowWidth="16905" windowHeight="13485" xr2:uid="{9E7B8A6A-42F7-4783-B41C-E02948B47874}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9E7B8A6A-42F7-4783-B41C-E02948B47874}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="42">
   <si>
     <t>Week 2</t>
   </si>
@@ -140,9 +140,6 @@
     <t>Added</t>
   </si>
   <si>
-    <t>Add some results to demo</t>
-  </si>
-  <si>
     <t>&lt;---extended Left</t>
   </si>
   <si>
@@ -159,6 +156,12 @@
   </si>
   <si>
     <t>Halow??? Long range WiFi</t>
+  </si>
+  <si>
+    <t>Some Results Available</t>
+  </si>
+  <si>
+    <t>Final Paper Review and Completion</t>
   </si>
 </sst>
 </file>
@@ -233,7 +236,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -347,6 +350,57 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -357,7 +411,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
@@ -387,6 +441,20 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="4" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="40% - Accent4" xfId="3" builtinId="43"/>
@@ -725,15 +793,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FA40F8A-DE14-4A53-9DE9-CC33AFA0ED4A}">
-  <dimension ref="B2:M64"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:M96"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="38.88671875" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D2" s="25" t="s">
         <v>30</v>
       </c>
@@ -741,7 +809,7 @@
         <v>46127</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
@@ -776,7 +844,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C4" s="19">
         <v>46115</v>
       </c>
@@ -811,7 +879,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>14</v>
       </c>
@@ -827,7 +895,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="8"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B6" s="17" t="s">
         <v>10</v>
       </c>
@@ -835,26 +903,26 @@
       <c r="E6" s="17"/>
       <c r="M6" s="10"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B7" s="17"/>
       <c r="E7" s="17"/>
       <c r="M7" s="10"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B8" s="17" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="24"/>
       <c r="M8" s="10"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B9" s="17" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="24"/>
       <c r="M9" s="10"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B10" s="17" t="s">
         <v>20</v>
       </c>
@@ -862,7 +930,7 @@
       <c r="F10" s="11"/>
       <c r="M10" s="10"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B11" s="17" t="s">
         <v>19</v>
       </c>
@@ -870,7 +938,7 @@
       <c r="G11" s="11"/>
       <c r="M11" s="10"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B12" s="17" t="s">
         <v>18</v>
       </c>
@@ -879,7 +947,7 @@
       <c r="H12" s="11"/>
       <c r="M12" s="10"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B13" s="17" t="s">
         <v>22</v>
       </c>
@@ -888,12 +956,12 @@
       <c r="I13" s="12"/>
       <c r="M13" s="10"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B14" s="17"/>
       <c r="E14" s="17"/>
       <c r="M14" s="10"/>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B15" s="17" t="s">
         <v>11</v>
       </c>
@@ -901,7 +969,7 @@
       <c r="H15" s="13"/>
       <c r="M15" s="10"/>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B16" s="17" t="s">
         <v>21</v>
       </c>
@@ -910,12 +978,12 @@
       <c r="J16" s="13"/>
       <c r="M16" s="10"/>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B17" s="17"/>
       <c r="E17" s="17"/>
       <c r="M17" s="10"/>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B18" s="17" t="s">
         <v>24</v>
       </c>
@@ -924,7 +992,7 @@
       <c r="J18" s="12"/>
       <c r="M18" s="10"/>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B19" s="17" t="s">
         <v>23</v>
       </c>
@@ -933,12 +1001,12 @@
       <c r="K19" s="12"/>
       <c r="M19" s="10"/>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B20" s="17"/>
       <c r="E20" s="17"/>
       <c r="M20" s="10"/>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B21" s="17" t="s">
         <v>12</v>
       </c>
@@ -947,7 +1015,7 @@
       <c r="L21" s="13"/>
       <c r="M21" s="10"/>
     </row>
-    <row r="22" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="18" t="s">
         <v>13</v>
       </c>
@@ -963,7 +1031,7 @@
       <c r="L22" s="14"/>
       <c r="M22" s="15"/>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B24" s="22" t="s">
         <v>25</v>
       </c>
@@ -972,25 +1040,25 @@
       </c>
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C25" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="3"/>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C26" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D26" s="4"/>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C27" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D27" s="2"/>
     </row>
-    <row r="29" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F29" s="25" t="s">
         <v>30</v>
       </c>
@@ -998,7 +1066,7 @@
         <v>46141</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C30" s="5" t="s">
         <v>9</v>
       </c>
@@ -1011,7 +1079,7 @@
       <c r="F30" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="G30" s="16" t="s">
+      <c r="G30" s="7" t="s">
         <v>2</v>
       </c>
       <c r="H30" s="7" t="s">
@@ -1033,7 +1101,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C31" s="19">
         <v>46115</v>
       </c>
@@ -1046,7 +1114,7 @@
       <c r="F31" s="20">
         <v>46136</v>
       </c>
-      <c r="G31" s="23">
+      <c r="G31" s="20">
         <v>46143</v>
       </c>
       <c r="H31" s="20">
@@ -1068,173 +1136,198 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B32" s="16" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="7"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="16"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
       <c r="M32" s="8"/>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B33" s="17" t="s">
         <v>10</v>
       </c>
       <c r="D33" s="9"/>
-      <c r="G33" s="17"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="17"/>
       <c r="M33" s="10"/>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B34" s="17"/>
-      <c r="G34" s="17"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="17"/>
       <c r="M34" s="10"/>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B35" s="17" t="s">
         <v>16</v>
       </c>
       <c r="E35" s="9"/>
-      <c r="G35" s="17"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="17"/>
       <c r="M35" s="10"/>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B36" s="17" t="s">
         <v>17</v>
       </c>
       <c r="E36" s="9"/>
-      <c r="G36" s="17"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="17"/>
       <c r="M36" s="10"/>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B37" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="F37" s="9"/>
-      <c r="G37" s="17"/>
+      <c r="F37" s="35"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="17"/>
       <c r="M37" s="10"/>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B38" s="17" t="s">
         <v>19</v>
       </c>
+      <c r="F38" s="34"/>
       <c r="G38" s="9" t="s">
         <v>31</v>
       </c>
+      <c r="H38" s="17"/>
       <c r="M38" s="10"/>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B39" s="17" t="s">
         <v>18</v>
       </c>
+      <c r="F39" s="34"/>
       <c r="G39" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H39" s="9"/>
+      <c r="H39" s="29"/>
       <c r="M39" s="10"/>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B40" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F40" s="12"/>
+      <c r="F40" s="36"/>
       <c r="G40" s="12"/>
-      <c r="H40" s="12" t="s">
-        <v>35</v>
+      <c r="H40" s="30" t="s">
+        <v>34</v>
       </c>
       <c r="M40" s="10"/>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B41" s="17"/>
-      <c r="G41" s="17"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="17"/>
       <c r="M41" s="10"/>
     </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B42" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="G42" s="17"/>
-      <c r="H42" s="13" t="s">
-        <v>34</v>
+      <c r="F42" s="34"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="31" t="s">
+        <v>40</v>
       </c>
       <c r="M42" s="10"/>
     </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B43" s="17" t="s">
         <v>21</v>
       </c>
+      <c r="F43" s="34"/>
       <c r="G43" s="9"/>
+      <c r="H43" s="17"/>
       <c r="I43" s="13" t="s">
         <v>31</v>
       </c>
       <c r="M43" s="10"/>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B44" s="17"/>
-      <c r="G44" s="17"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="17"/>
       <c r="M44" s="10"/>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B45" s="17" t="s">
         <v>24</v>
       </c>
+      <c r="F45" s="34"/>
       <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
+      <c r="H45" s="30"/>
       <c r="I45" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J45" s="12"/>
       <c r="M45" s="10"/>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B46" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="G46" s="17"/>
-      <c r="H46" s="12"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="30"/>
       <c r="I46" s="12"/>
       <c r="J46" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M46" s="10"/>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B47" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="G47" s="17"/>
+      <c r="F47" s="34"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="17"/>
       <c r="K47" s="3" t="s">
         <v>33</v>
       </c>
       <c r="L47" s="3"/>
       <c r="M47" s="10"/>
     </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B48" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G48" s="17"/>
+      <c r="F48" s="34"/>
+      <c r="G48" s="32"/>
+      <c r="H48" s="17"/>
       <c r="K48" s="13"/>
       <c r="L48" s="13"/>
       <c r="M48" s="10"/>
     </row>
-    <row r="49" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C49" s="14"/>
       <c r="D49" s="14"/>
       <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="18"/>
-      <c r="H49" s="14"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="18"/>
       <c r="I49" s="14"/>
       <c r="J49" s="14"/>
       <c r="K49" s="14"/>
@@ -1243,7 +1336,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B51" s="22" t="s">
         <v>25</v>
       </c>
@@ -1252,52 +1345,410 @@
       </c>
       <c r="D51" s="1"/>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C52" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D52" s="3"/>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C53" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D53" s="4"/>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C54" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D54" s="2"/>
     </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B61" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B61" t="s">
+    <row r="62" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
+    <row r="63" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B63" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
+    <row r="64" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
+    <row r="70" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F70" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="G70" s="26">
+        <v>46150</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C71" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H71" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I71" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J71" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K71" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L71" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="M71" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C72" s="19">
+        <v>46115</v>
+      </c>
+      <c r="D72" s="20">
+        <v>46122</v>
+      </c>
+      <c r="E72" s="20">
+        <v>46129</v>
+      </c>
+      <c r="F72" s="20">
+        <v>46136</v>
+      </c>
+      <c r="G72" s="20">
+        <v>46143</v>
+      </c>
+      <c r="H72" s="20">
+        <v>46150</v>
+      </c>
+      <c r="I72" s="20">
+        <v>46157</v>
+      </c>
+      <c r="J72" s="20">
+        <v>46164</v>
+      </c>
+      <c r="K72" s="20">
+        <v>46171</v>
+      </c>
+      <c r="L72" s="20">
+        <v>46178</v>
+      </c>
+      <c r="M72" s="21">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B73" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C73" s="6"/>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="33"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="16"/>
+      <c r="I73" s="5"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="8"/>
+    </row>
+    <row r="74" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B74" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D74" s="9"/>
+      <c r="F74" s="34"/>
+      <c r="G74" s="32"/>
+      <c r="H74" s="17"/>
+      <c r="I74" s="27"/>
+      <c r="J74" s="32"/>
+      <c r="K74" s="32"/>
+      <c r="L74" s="32"/>
+      <c r="M74" s="10"/>
+    </row>
+    <row r="75" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B75" s="17"/>
+      <c r="F75" s="34"/>
+      <c r="G75" s="32"/>
+      <c r="H75" s="17"/>
+      <c r="I75" s="27"/>
+      <c r="J75" s="32"/>
+      <c r="K75" s="32"/>
+      <c r="L75" s="32"/>
+      <c r="M75" s="10"/>
+    </row>
+    <row r="76" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B76" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="E76" s="9"/>
+      <c r="F76" s="34"/>
+      <c r="G76" s="32"/>
+      <c r="H76" s="17"/>
+      <c r="I76" s="27"/>
+      <c r="J76" s="32"/>
+      <c r="K76" s="32"/>
+      <c r="L76" s="32"/>
+      <c r="M76" s="10"/>
+    </row>
+    <row r="77" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B77" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E77" s="9"/>
+      <c r="F77" s="34"/>
+      <c r="G77" s="32"/>
+      <c r="H77" s="17"/>
+      <c r="I77" s="27"/>
+      <c r="J77" s="32"/>
+      <c r="K77" s="32"/>
+      <c r="L77" s="32"/>
+      <c r="M77" s="10"/>
+    </row>
+    <row r="78" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B78" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F78" s="35"/>
+      <c r="G78" s="32"/>
+      <c r="H78" s="17"/>
+      <c r="I78" s="27"/>
+      <c r="J78" s="32"/>
+      <c r="K78" s="32"/>
+      <c r="L78" s="32"/>
+      <c r="M78" s="10"/>
+    </row>
+    <row r="79" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B79" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="F79" s="34"/>
+      <c r="G79" s="9"/>
+      <c r="H79" s="17"/>
+      <c r="I79" s="27"/>
+      <c r="J79" s="32"/>
+      <c r="K79" s="32"/>
+      <c r="L79" s="32"/>
+      <c r="M79" s="10"/>
+    </row>
+    <row r="80" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B80" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F80" s="34"/>
+      <c r="G80" s="9"/>
+      <c r="H80" s="29"/>
+      <c r="I80" s="27"/>
+      <c r="J80" s="32"/>
+      <c r="K80" s="32"/>
+      <c r="L80" s="32"/>
+      <c r="M80" s="10"/>
+    </row>
+    <row r="81" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B81" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F81" s="36"/>
+      <c r="G81" s="12"/>
+      <c r="H81" s="30"/>
+      <c r="I81" s="38"/>
+      <c r="J81" s="32"/>
+      <c r="K81" s="32"/>
+      <c r="L81" s="32"/>
+      <c r="M81" s="10"/>
+    </row>
+    <row r="82" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B82" s="17"/>
+      <c r="F82" s="34"/>
+      <c r="G82" s="32"/>
+      <c r="H82" s="17"/>
+      <c r="I82" s="27"/>
+      <c r="J82" s="32"/>
+      <c r="K82" s="32"/>
+      <c r="L82" s="32"/>
+      <c r="M82" s="10"/>
+    </row>
+    <row r="83" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B83" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F83" s="34"/>
+      <c r="G83" s="32"/>
+      <c r="H83" s="31" t="s">
         <v>40</v>
       </c>
+      <c r="I83" s="27"/>
+      <c r="J83" s="32"/>
+      <c r="K83" s="32"/>
+      <c r="L83" s="32"/>
+      <c r="M83" s="10"/>
+    </row>
+    <row r="84" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B84" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F84" s="34"/>
+      <c r="G84" s="9"/>
+      <c r="H84" s="17"/>
+      <c r="I84" s="39"/>
+      <c r="J84" s="32"/>
+      <c r="K84" s="32"/>
+      <c r="L84" s="32"/>
+      <c r="M84" s="10"/>
+    </row>
+    <row r="85" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B85" s="17"/>
+      <c r="F85" s="34"/>
+      <c r="G85" s="32"/>
+      <c r="H85" s="17"/>
+      <c r="I85" s="27"/>
+      <c r="J85" s="32"/>
+      <c r="K85" s="32"/>
+      <c r="L85" s="32"/>
+      <c r="M85" s="10"/>
+    </row>
+    <row r="86" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B86" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F86" s="34"/>
+      <c r="G86" s="12"/>
+      <c r="H86" s="30"/>
+      <c r="I86" s="40"/>
+      <c r="J86" s="12"/>
+      <c r="K86" s="32"/>
+      <c r="L86" s="32"/>
+      <c r="M86" s="10"/>
+    </row>
+    <row r="87" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B87" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F87" s="34"/>
+      <c r="G87" s="32"/>
+      <c r="H87" s="30"/>
+      <c r="I87" s="40"/>
+      <c r="J87" s="12"/>
+      <c r="K87" s="32"/>
+      <c r="L87" s="32"/>
+      <c r="M87" s="10"/>
+    </row>
+    <row r="88" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B88" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="F88" s="34"/>
+      <c r="G88" s="32"/>
+      <c r="H88" s="17"/>
+      <c r="I88" s="27"/>
+      <c r="J88" s="32"/>
+      <c r="K88" s="12"/>
+      <c r="L88" s="12"/>
+      <c r="M88" s="10"/>
+    </row>
+    <row r="89" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B89" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F89" s="34"/>
+      <c r="G89" s="32"/>
+      <c r="H89" s="17"/>
+      <c r="I89" s="27"/>
+      <c r="J89" s="32"/>
+      <c r="K89" s="11"/>
+      <c r="L89" s="11"/>
+      <c r="M89" s="10"/>
+    </row>
+    <row r="90" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B90" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F90" s="34"/>
+      <c r="G90" s="32"/>
+      <c r="H90" s="17"/>
+      <c r="I90" s="27"/>
+      <c r="J90" s="32"/>
+      <c r="K90" s="13"/>
+      <c r="L90" s="13"/>
+      <c r="M90" s="10"/>
+    </row>
+    <row r="91" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B91" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C91" s="14"/>
+      <c r="D91" s="14"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="37"/>
+      <c r="G91" s="14"/>
+      <c r="H91" s="18"/>
+      <c r="I91" s="28"/>
+      <c r="J91" s="14"/>
+      <c r="K91" s="14"/>
+      <c r="L91" s="14"/>
+      <c r="M91" s="15"/>
+    </row>
+    <row r="93" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B93" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D93" s="1"/>
+    </row>
+    <row r="94" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C94" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D94" s="3"/>
+    </row>
+    <row r="95" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C95" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D95" s="4"/>
+    </row>
+    <row r="96" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C96" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D96" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>